<commit_message>
Add group-wide summary CSV generator
Add generate_summaries.py, which reads the same directory of Research Record
spreadsheets and writes aggregated CSVs:

- presentations.csv: every talk/poster/seminar
- publications.csv: every paper/note
- conferences.csv: unique conferences attended (attendees, years, counts)
- schools.csv: unique schools/lecture courses attended

Conferences and schools are derived from the Presentations tab (no separate
attendance field exists): Lecture-typed entries and school/academy/tutorial
venues are schools, the rest conferences; venues are grouped by series so a
trailing year is collapsed. Also add a school sample record, .gitignore, a
demo summaries/ output, and README docs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019AZa5wYxJDkZMK7fkTTU4S
</commit_message>
<xml_diff>
--- a/sample_data/CarolineDavis_Info.xlsx
+++ b/sample_data/CarolineDavis_Info.xlsx
@@ -4917,15 +4917,45 @@
       <c r="I10" s="18" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>US Particle Accelerator School 2025</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Knoxville, TN</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Attendee — accelerator physics</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="19" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="n"/>

</xml_diff>

<commit_message>
Add group-wide summary CSV generator (#2)
Add generate_summaries.py, which reads the same directory of Research Record
spreadsheets and writes aggregated CSVs:

- presentations.csv: every talk/poster/seminar
- publications.csv: every paper/note
- conferences.csv: unique conferences attended (attendees, years, counts)
- schools.csv: unique schools/lecture courses attended

Conferences and schools are derived from the Presentations tab (no separate
attendance field exists): Lecture-typed entries and school/academy/tutorial
venues are schools, the rest conferences; venues are grouped by series so a
trailing year is collapsed. Also add a school sample record, .gitignore, a
demo summaries/ output, and README docs.


Claude-Session: https://claude.ai/code/session_019AZa5wYxJDkZMK7fkTTU4S

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/CarolineDavis_Info.xlsx
+++ b/sample_data/CarolineDavis_Info.xlsx
@@ -4917,15 +4917,45 @@
       <c r="I10" s="18" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>US Particle Accelerator School 2025</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Knoxville, TN</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Attendee — accelerator physics</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="19" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="n"/>

</xml_diff>